<commit_message>
agregando fechas al lead
</commit_message>
<xml_diff>
--- a/modelado/modelado/importarlead2.xlsx
+++ b/modelado/modelado/importarlead2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\tradecar\modelado\modelado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97DDAB9D-1F8A-4F27-95B0-2FFB49F68F57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{993BF833-E5E6-44AA-B788-FA2200BC6165}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2B6254AE-AAC2-B142-8A5F-DD575D2DDDDB}"/>
   </bookViews>
@@ -1612,7 +1612,7 @@
         <v>75000</v>
       </c>
       <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
+      <c r="K5" s="2"/>
       <c r="L5" s="3"/>
       <c r="M5" s="2">
         <v>1</v>
@@ -1793,7 +1793,7 @@
         <v>94000</v>
       </c>
       <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
+      <c r="K10" s="2"/>
       <c r="L10" s="3"/>
       <c r="M10" s="2">
         <v>1</v>
@@ -1976,7 +1976,7 @@
         <v>78000</v>
       </c>
       <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
+      <c r="K15" s="2"/>
       <c r="L15" s="3"/>
       <c r="M15" s="2">
         <v>1</v>
@@ -2085,7 +2085,7 @@
         <v>7000</v>
       </c>
       <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
+      <c r="K18" s="2"/>
       <c r="L18" s="3"/>
       <c r="M18" s="2">
         <v>1</v>
@@ -2194,7 +2194,7 @@
         <v>200</v>
       </c>
       <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
+      <c r="K21" s="2"/>
       <c r="L21" s="3"/>
       <c r="M21" s="2">
         <v>1</v>
@@ -2340,7 +2340,7 @@
         <v>70000</v>
       </c>
       <c r="J25" s="3"/>
-      <c r="K25" s="3"/>
+      <c r="K25" s="2"/>
       <c r="L25" s="3"/>
       <c r="M25" s="2">
         <v>1</v>
@@ -2486,7 +2486,7 @@
         <v>230000</v>
       </c>
       <c r="J29" s="3"/>
-      <c r="K29" s="3"/>
+      <c r="K29" s="2"/>
       <c r="L29" s="3"/>
       <c r="M29" s="2">
         <v>1</v>
@@ -2632,7 +2632,7 @@
         <v>204</v>
       </c>
       <c r="J33" s="3"/>
-      <c r="K33" s="3"/>
+      <c r="K33" s="2"/>
       <c r="L33" s="3"/>
       <c r="M33" s="2">
         <v>1</v>
@@ -2667,7 +2667,7 @@
         <v>34500</v>
       </c>
       <c r="J34" s="3"/>
-      <c r="K34" s="3"/>
+      <c r="K34" s="2"/>
       <c r="L34" s="3"/>
       <c r="M34" s="2">
         <v>1</v>
@@ -2702,7 +2702,7 @@
         <v>150000</v>
       </c>
       <c r="J35" s="3"/>
-      <c r="K35" s="3"/>
+      <c r="K35" s="2"/>
       <c r="L35" s="3"/>
       <c r="M35" s="2">
         <v>1</v>
@@ -2737,7 +2737,7 @@
         <v>78000</v>
       </c>
       <c r="J36" s="3"/>
-      <c r="K36" s="3"/>
+      <c r="K36" s="2"/>
       <c r="L36" s="3"/>
       <c r="M36" s="2">
         <v>1</v>
@@ -2772,7 +2772,7 @@
         <v>205</v>
       </c>
       <c r="J37" s="3"/>
-      <c r="K37" s="3"/>
+      <c r="K37" s="2"/>
       <c r="L37" s="3"/>
       <c r="M37" s="2">
         <v>1</v>
@@ -2807,7 +2807,7 @@
         <v>125</v>
       </c>
       <c r="J38" s="3"/>
-      <c r="K38" s="3"/>
+      <c r="K38" s="2"/>
       <c r="L38" s="3"/>
       <c r="M38" s="2">
         <v>1</v>
@@ -2916,7 +2916,7 @@
         <v>206</v>
       </c>
       <c r="J41" s="3"/>
-      <c r="K41" s="3"/>
+      <c r="K41" s="2"/>
       <c r="L41" s="3"/>
       <c r="M41" s="2">
         <v>1</v>
@@ -2951,7 +2951,7 @@
         <v>136000</v>
       </c>
       <c r="J42" s="3"/>
-      <c r="K42" s="3"/>
+      <c r="K42" s="2"/>
       <c r="L42" s="3"/>
       <c r="M42" s="2">
         <v>1</v>
@@ -3023,7 +3023,7 @@
         <v>145000</v>
       </c>
       <c r="J44" s="3"/>
-      <c r="K44" s="3"/>
+      <c r="K44" s="2"/>
       <c r="L44" s="3"/>
       <c r="M44" s="2">
         <v>1</v>
@@ -3058,7 +3058,7 @@
         <v>166500</v>
       </c>
       <c r="J45" s="3"/>
-      <c r="K45" s="3"/>
+      <c r="K45" s="2"/>
       <c r="L45" s="3"/>
       <c r="M45" s="2">
         <v>1</v>
@@ -3204,7 +3204,7 @@
         <v>208</v>
       </c>
       <c r="J49" s="3"/>
-      <c r="K49" s="3"/>
+      <c r="K49" s="2"/>
       <c r="L49" s="3"/>
       <c r="M49" s="2">
         <v>1</v>
@@ -3350,7 +3350,7 @@
         <v>209</v>
       </c>
       <c r="J53" s="3"/>
-      <c r="K53" s="3"/>
+      <c r="K53" s="2"/>
       <c r="L53" s="3"/>
       <c r="M53" s="2">
         <v>1</v>
@@ -3385,7 +3385,7 @@
         <v>175000</v>
       </c>
       <c r="J54" s="3"/>
-      <c r="K54" s="3"/>
+      <c r="K54" s="2"/>
       <c r="L54" s="3"/>
       <c r="M54" s="2">
         <v>1</v>
@@ -3457,7 +3457,7 @@
         <v>123000</v>
       </c>
       <c r="J56" s="3"/>
-      <c r="K56" s="3"/>
+      <c r="K56" s="2"/>
       <c r="L56" s="3"/>
       <c r="M56" s="2">
         <v>1</v>
@@ -3529,7 +3529,7 @@
         <v>31996</v>
       </c>
       <c r="J58" s="3"/>
-      <c r="K58" s="3"/>
+      <c r="K58" s="2"/>
       <c r="L58" s="3"/>
       <c r="M58" s="2">
         <v>1</v>
@@ -3603,7 +3603,7 @@
       <c r="J60" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="K60" s="6"/>
+      <c r="K60" s="2"/>
       <c r="L60" s="6"/>
       <c r="M60" s="2">
         <v>1</v>
@@ -3640,7 +3640,7 @@
       <c r="J61" s="9" t="s">
         <v>272</v>
       </c>
-      <c r="K61" s="9"/>
+      <c r="K61" s="2"/>
       <c r="L61" s="9"/>
       <c r="M61" s="2">
         <v>1</v>
@@ -3677,7 +3677,7 @@
       <c r="J62" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="K62" s="6"/>
+      <c r="K62" s="2"/>
       <c r="L62" s="6"/>
       <c r="M62" s="2">
         <v>1</v>
@@ -3714,7 +3714,7 @@
       <c r="J63" s="9" t="s">
         <v>274</v>
       </c>
-      <c r="K63" s="9"/>
+      <c r="K63" s="2"/>
       <c r="L63" s="9"/>
       <c r="M63" s="2">
         <v>1</v>
@@ -3751,7 +3751,7 @@
       <c r="J64" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="K64" s="6"/>
+      <c r="K64" s="2"/>
       <c r="L64" s="6"/>
       <c r="M64" s="2">
         <v>1</v>
@@ -3788,7 +3788,7 @@
       <c r="J65" s="9" t="s">
         <v>275</v>
       </c>
-      <c r="K65" s="9"/>
+      <c r="K65" s="2"/>
       <c r="L65" s="9"/>
       <c r="M65" s="2">
         <v>1</v>

</xml_diff>